<commit_message>
feat: support uint64 game values #370
- Expand HP, MP, money, experience, damage, and marketplace prices to 64-bit values
- Add client amount encoding, protocol updates, database migrations, and integration coverage
- Rename mob AI strategies and add inert behavior
- Settle multipart mobs and their rewards independently
- Harden Lua integer and coroutine handling
</commit_message>
<xml_diff>
--- a/resources/table/enum.mob.xlsx
+++ b/resources/table/enum.mob.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cshyeon\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021F4642-3192-44F9-B548-7DD7386CD515}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350AC582-CA3A-494C-A8BA-D979A94144E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="MOB_SIZE" sheetId="1" r:id="rId1"/>
@@ -26,28 +26,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>NONE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>COUNTER</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CONTAINMENT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>RUN_AWAY</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>NO_MOVE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>SMALL</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -61,6 +49,22 @@
   </si>
   <si>
     <t>SMALL | LARGE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RETALIATE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGGRESSIVE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>STATIONARY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>INERT</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -466,7 +470,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1">
         <v>1</v>
@@ -474,7 +478,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1">
         <v>2</v>
@@ -482,10 +486,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -496,7 +500,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D978953-EF9D-43EE-AFAC-388FB72E496C}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.375" style="1" customWidth="1"/>
@@ -513,7 +517,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -521,7 +525,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -529,7 +533,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -537,10 +541,18 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add resist system and integration tests
- Add RESIST enum and mob resist model fields
- Apply PHYSICAL/MAGIC resist in damage calculation
- Gate SPELL/MOVE/status effects in spell helpers
- Add atomic server helpers for parts and resist checks
- Register mob_parts_test and resist_test suites
</commit_message>
<xml_diff>
--- a/resources/table/enum.mob.xlsx
+++ b/resources/table/enum.mob.xlsx
@@ -8,64 +8,77 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350AC582-CA3A-494C-A8BA-D979A94144E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9816C3A9-5501-4DF8-996A-19F8B803BEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MOB_SIZE" sheetId="1" r:id="rId1"/>
     <sheet name="MOB_ATTACK_TYPE" sheetId="2" r:id="rId2"/>
+    <sheet name="RESIST" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>NONE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RETALIATE</t>
+  </si>
+  <si>
+    <t>AGGRESSIVE</t>
   </si>
   <si>
     <t>RUN_AWAY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>STATIONARY</t>
+  </si>
+  <si>
+    <t>INERT</t>
   </si>
   <si>
     <t>SMALL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>LARGE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>ALL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>SMALL | LARGE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RETALIATE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>AGGRESSIVE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>STATIONARY</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>INERT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PHYSICAL</t>
+  </si>
+  <si>
+    <t>MAGIC</t>
+  </si>
+  <si>
+    <t>SPELL</t>
+  </si>
+  <si>
+    <t>MOVE</t>
+  </si>
+  <si>
+    <t>PARALYSIS</t>
+  </si>
+  <si>
+    <t>POISON</t>
+  </si>
+  <si>
+    <t>DESPAIR</t>
+  </si>
+  <si>
+    <t>CURSE</t>
+  </si>
+  <si>
+    <t>BLIND</t>
   </si>
 </sst>
 </file>
@@ -459,18 +472,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39046541-05ED-4D1B-A199-7B090CD6E48E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="12.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="1"/>
+    <col min="3" max="3" width="9" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1">
         <v>1</v>
@@ -478,7 +492,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1">
         <v>2</v>
@@ -486,10 +500,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -499,12 +513,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D978953-EF9D-43EE-AFAC-388FB72E496C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.375" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="9" style="1"/>
+    <col min="2" max="2" width="9" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -517,7 +532,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -525,7 +540,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -533,7 +548,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -541,7 +556,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
@@ -549,7 +564,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1">
         <v>5</v>
@@ -559,4 +574,90 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>